<commit_message>
VIs and Data Iterations Organized
</commit_message>
<xml_diff>
--- a/system_development/Damascus/V0.5.0/software development/Event Camera/v0.2/Event Camera Test Parameters.xlsx
+++ b/system_development/Damascus/V0.5.0/software development/Event Camera/v0.2/Event Camera Test Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\LPBF-Observer\system_development\Damascus\V0.5.0\software development\Event Camera\v0.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78AE2D1-D819-4E8A-B33D-EFE5D3CD0087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16407D73-4654-4CBC-A7BA-3689158565F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="89">
   <si>
     <t>Date</t>
   </si>
@@ -267,6 +266,42 @@
   <si>
     <t>spatter looks like a flame</t>
   </si>
+  <si>
+    <t>Shade 5</t>
+  </si>
+  <si>
+    <t>Shade 9</t>
+  </si>
+  <si>
+    <t>Shade 12</t>
+  </si>
+  <si>
+    <t>Test_2</t>
+  </si>
+  <si>
+    <t>Test_1</t>
+  </si>
+  <si>
+    <t>Test_3</t>
+  </si>
+  <si>
+    <t>Test_4</t>
+  </si>
+  <si>
+    <t>no shade</t>
+  </si>
+  <si>
+    <t>4-line scan</t>
+  </si>
+  <si>
+    <t>small circle</t>
+  </si>
+  <si>
+    <t>(not complete)</t>
+  </si>
+  <si>
+    <t>"</t>
+  </si>
 </sst>
 </file>
 
@@ -275,7 +310,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -314,6 +349,11 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -404,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -505,6 +545,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -833,8 +876,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{32870E6A-1628-4B15-B791-04B0D0E7C0CE}" name="Table1" displayName="Table1" ref="B3:P44" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
-  <autoFilter ref="B3:P44" xr:uid="{32870E6A-1628-4B15-B791-04B0D0E7C0CE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{32870E6A-1628-4B15-B791-04B0D0E7C0CE}" name="Table1" displayName="Table1" ref="B3:P56" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="B3:P56" xr:uid="{32870E6A-1628-4B15-B791-04B0D0E7C0CE}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{EF9C8B83-DF18-4080-80FA-82B3ABAB5E82}" name="test" dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{0B6F9DE2-0A0C-4916-BC37-A368355A29D4}" name="Defocus" dataDxfId="13"/>
@@ -1057,7 +1100,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:AD1010"/>
+  <dimension ref="B1:AD1022"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.44140625" customWidth="1"/>
@@ -1250,7 +1293,7 @@
     </row>
     <row r="5" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B5" s="11">
-        <f t="shared" ref="B5:B44" si="0">SUM(B4 + 1)</f>
+        <f t="shared" ref="B5:B56" si="0">SUM(B4 + 1)</f>
         <v>2</v>
       </c>
       <c r="C5" s="2">
@@ -2651,13 +2694,23 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
+      <c r="C33" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D33" s="3">
+        <v>75</v>
+      </c>
+      <c r="E33" s="3">
+        <v>300</v>
+      </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
+      <c r="H33" s="3">
+        <v>0</v>
+      </c>
+      <c r="I33" s="3">
+        <v>0</v>
+      </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3" t="s">
@@ -2694,13 +2747,23 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
+      <c r="C34" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D34" s="3">
+        <v>75</v>
+      </c>
+      <c r="E34" s="3">
+        <v>300</v>
+      </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
+      <c r="H34" s="3">
+        <v>0</v>
+      </c>
+      <c r="I34" s="3">
+        <v>0</v>
+      </c>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3" t="s">
@@ -2738,13 +2801,23 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
+      <c r="C35" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D35" s="3">
+        <v>75</v>
+      </c>
+      <c r="E35" s="3">
+        <v>300</v>
+      </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
+      <c r="H35" s="3">
+        <v>0</v>
+      </c>
+      <c r="I35" s="3">
+        <v>0</v>
+      </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3" t="s">
@@ -2782,13 +2855,23 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
+      <c r="C36" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D36" s="3">
+        <v>75</v>
+      </c>
+      <c r="E36" s="3">
+        <v>300</v>
+      </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
+      <c r="H36" s="3">
+        <v>0</v>
+      </c>
+      <c r="I36" s="3">
+        <v>0</v>
+      </c>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3" t="s">
@@ -2826,13 +2909,23 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
+      <c r="C37" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D37" s="3">
+        <v>75</v>
+      </c>
+      <c r="E37" s="3">
+        <v>300</v>
+      </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
+      <c r="H37" s="3">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3">
+        <v>0</v>
+      </c>
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3" t="s">
@@ -2870,13 +2963,23 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
+      <c r="C38" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D38" s="3">
+        <v>75</v>
+      </c>
+      <c r="E38" s="3">
+        <v>300</v>
+      </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
+      <c r="H38" s="3">
+        <v>0</v>
+      </c>
+      <c r="I38" s="3">
+        <v>0</v>
+      </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3" t="s">
@@ -2916,13 +3019,23 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
+      <c r="C39" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D39" s="3">
+        <v>75</v>
+      </c>
+      <c r="E39" s="3">
+        <v>300</v>
+      </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
+      <c r="H39" s="3">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3">
+        <v>0</v>
+      </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3" t="s">
@@ -2958,13 +3071,23 @@
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
+      <c r="C40" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D40" s="3">
+        <v>75</v>
+      </c>
+      <c r="E40" s="3">
+        <v>300</v>
+      </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
-      <c r="I40" s="3"/>
+      <c r="H40" s="3">
+        <v>0</v>
+      </c>
+      <c r="I40" s="3">
+        <v>0</v>
+      </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3" t="s">
@@ -3000,13 +3123,23 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
+      <c r="C41" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D41" s="3">
+        <v>75</v>
+      </c>
+      <c r="E41" s="3">
+        <v>300</v>
+      </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
+      <c r="H41" s="3">
+        <v>0</v>
+      </c>
+      <c r="I41" s="3">
+        <v>0</v>
+      </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3" t="s">
@@ -3044,20 +3177,36 @@
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
+      <c r="C42" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D42" s="3">
+        <v>75</v>
+      </c>
+      <c r="E42" s="3">
+        <v>300</v>
+      </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
+      <c r="H42" s="3">
+        <v>0</v>
+      </c>
+      <c r="I42" s="3">
+        <v>0</v>
+      </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
-      <c r="M42" s="15"/>
-      <c r="N42" s="25"/>
-      <c r="O42" s="1"/>
-      <c r="P42" s="1"/>
+      <c r="L42" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="M42" s="28">
+        <v>46297</v>
+      </c>
+      <c r="N42" s="27">
+        <v>2</v>
+      </c>
+      <c r="O42" s="36"/>
+      <c r="P42" s="36"/>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
@@ -3078,18 +3227,34 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
+      <c r="C43" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D43" s="3">
+        <v>75</v>
+      </c>
+      <c r="E43" s="3">
+        <v>300</v>
+      </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
-      <c r="H43" s="3"/>
-      <c r="I43" s="3"/>
+      <c r="H43" s="3">
+        <v>0</v>
+      </c>
+      <c r="I43" s="3">
+        <v>0</v>
+      </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3"/>
-      <c r="L43" s="3"/>
-      <c r="M43" s="15"/>
-      <c r="N43" s="25"/>
+      <c r="L43" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="M43" s="15">
+        <v>46296</v>
+      </c>
+      <c r="N43" s="25">
+        <v>3</v>
+      </c>
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
@@ -3112,19 +3277,33 @@
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
+      <c r="C44" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D44" s="3">
+        <v>75</v>
+      </c>
+      <c r="E44" s="3">
+        <v>300</v>
+      </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
-      <c r="I44" s="3"/>
+      <c r="H44" s="3">
+        <v>0</v>
+      </c>
+      <c r="I44" s="3">
+        <v>0</v>
+      </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
-      <c r="M44" s="15"/>
+      <c r="L44" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="M44" s="15">
+        <v>46296</v>
+      </c>
       <c r="N44" s="25"/>
-      <c r="O44" s="20"/>
+      <c r="O44" s="1"/>
       <c r="P44" s="1"/>
       <c r="Q44" s="1"/>
       <c r="R44" s="1"/>
@@ -3142,19 +3321,36 @@
       <c r="AD44" s="1"/>
     </row>
     <row r="45" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B45" s="11"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
+      <c r="B45" s="11">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="C45" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D45" s="3">
+        <v>75</v>
+      </c>
+      <c r="E45" s="3">
+        <v>300</v>
+      </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
-      <c r="I45" s="3"/>
+      <c r="H45" s="3">
+        <v>0</v>
+      </c>
+      <c r="I45" s="3">
+        <v>0</v>
+      </c>
       <c r="J45" s="3"/>
       <c r="K45" s="3"/>
-      <c r="L45" s="3"/>
-      <c r="M45" s="15"/>
-      <c r="N45" s="23"/>
+      <c r="L45" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="M45" s="15">
+        <v>46296</v>
+      </c>
+      <c r="N45" s="25"/>
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
@@ -3169,23 +3365,40 @@
       <c r="Z45" s="1"/>
       <c r="AA45" s="1"/>
       <c r="AB45" s="1"/>
+      <c r="AC45" s="1"/>
+      <c r="AD45" s="1"/>
     </row>
     <row r="46" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B46" s="11"/>
-      <c r="C46" s="21" t="s">
+      <c r="B46" s="11">
+        <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
+      <c r="C46" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D46" s="3">
+        <v>75</v>
+      </c>
+      <c r="E46" s="3">
+        <v>300</v>
+      </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
+      <c r="H46" s="3">
+        <v>0</v>
+      </c>
+      <c r="I46" s="3">
+        <v>0</v>
+      </c>
       <c r="J46" s="3"/>
       <c r="K46" s="3"/>
-      <c r="L46" s="3"/>
-      <c r="M46" s="15"/>
-      <c r="N46" s="23"/>
+      <c r="L46" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M46" s="15">
+        <v>46296</v>
+      </c>
+      <c r="N46" s="25"/>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
@@ -3200,21 +3413,40 @@
       <c r="Z46" s="1"/>
       <c r="AA46" s="1"/>
       <c r="AB46" s="1"/>
+      <c r="AC46" s="1"/>
+      <c r="AD46" s="1"/>
     </row>
     <row r="47" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B47" s="11"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
+      <c r="B47" s="11">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C47" s="2">
+        <v>5.8730000000000002</v>
+      </c>
+      <c r="D47" s="3">
+        <v>75</v>
+      </c>
+      <c r="E47" s="3">
+        <v>300</v>
+      </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
+      <c r="H47" s="3">
+        <v>0</v>
+      </c>
+      <c r="I47" s="3">
+        <v>0</v>
+      </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
-      <c r="L47" s="3"/>
-      <c r="M47" s="15"/>
-      <c r="N47" s="23"/>
+      <c r="L47" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M47" s="15">
+        <v>46296</v>
+      </c>
+      <c r="N47" s="25"/>
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
@@ -3229,9 +3461,14 @@
       <c r="Z47" s="1"/>
       <c r="AA47" s="1"/>
       <c r="AB47" s="1"/>
+      <c r="AC47" s="1"/>
+      <c r="AD47" s="1"/>
     </row>
     <row r="48" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B48" s="11"/>
+      <c r="B48" s="11">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
@@ -3241,10 +3478,18 @@
       <c r="I48" s="3"/>
       <c r="J48" s="3"/>
       <c r="K48" s="3"/>
-      <c r="L48" s="3"/>
-      <c r="M48" s="15"/>
-      <c r="N48" s="23"/>
-      <c r="O48" s="1"/>
+      <c r="L48" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="M48" s="28">
+        <v>46296</v>
+      </c>
+      <c r="N48" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="O48" s="1" t="s">
+        <v>85</v>
+      </c>
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
       <c r="R48" s="1"/>
@@ -3258,9 +3503,14 @@
       <c r="Z48" s="1"/>
       <c r="AA48" s="1"/>
       <c r="AB48" s="1"/>
-    </row>
-    <row r="49" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B49" s="11"/>
+      <c r="AC48" s="1"/>
+      <c r="AD48" s="1"/>
+    </row>
+    <row r="49" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B49" s="11">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
@@ -3270,10 +3520,18 @@
       <c r="I49" s="3"/>
       <c r="J49" s="3"/>
       <c r="K49" s="3"/>
-      <c r="L49" s="3"/>
-      <c r="M49" s="15"/>
-      <c r="N49" s="23"/>
-      <c r="O49" s="1"/>
+      <c r="L49" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="M49" s="15">
+        <v>46296</v>
+      </c>
+      <c r="N49" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="O49" s="1" t="s">
+        <v>86</v>
+      </c>
       <c r="P49" s="1"/>
       <c r="Q49" s="1"/>
       <c r="R49" s="1"/>
@@ -3287,9 +3545,14 @@
       <c r="Z49" s="1"/>
       <c r="AA49" s="1"/>
       <c r="AB49" s="1"/>
-    </row>
-    <row r="50" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B50" s="11"/>
+      <c r="AC49" s="1"/>
+      <c r="AD49" s="1"/>
+    </row>
+    <row r="50" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B50" s="11">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
@@ -3299,10 +3562,18 @@
       <c r="I50" s="3"/>
       <c r="J50" s="3"/>
       <c r="K50" s="3"/>
-      <c r="L50" s="3"/>
-      <c r="M50" s="15"/>
-      <c r="N50" s="23"/>
-      <c r="O50" s="1"/>
+      <c r="L50" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="M50" s="15">
+        <v>46296</v>
+      </c>
+      <c r="N50" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="O50" s="1" t="s">
+        <v>87</v>
+      </c>
       <c r="P50" s="1"/>
       <c r="Q50" s="1"/>
       <c r="R50" s="1"/>
@@ -3316,9 +3587,14 @@
       <c r="Z50" s="1"/>
       <c r="AA50" s="1"/>
       <c r="AB50" s="1"/>
-    </row>
-    <row r="51" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B51" s="11"/>
+      <c r="AC50" s="1"/>
+      <c r="AD50" s="1"/>
+    </row>
+    <row r="51" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B51" s="11">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
@@ -3328,10 +3604,18 @@
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
       <c r="K51" s="3"/>
-      <c r="L51" s="3"/>
-      <c r="M51" s="15"/>
-      <c r="N51" s="23"/>
-      <c r="O51" s="1"/>
+      <c r="L51" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M51" s="15">
+        <v>46296</v>
+      </c>
+      <c r="N51" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="O51" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
       <c r="R51" s="1"/>
@@ -3345,9 +3629,14 @@
       <c r="Z51" s="1"/>
       <c r="AA51" s="1"/>
       <c r="AB51" s="1"/>
-    </row>
-    <row r="52" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B52" s="11"/>
+      <c r="AC51" s="1"/>
+      <c r="AD51" s="1"/>
+    </row>
+    <row r="52" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B52" s="11">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
@@ -3359,7 +3648,7 @@
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="15"/>
-      <c r="N52" s="23"/>
+      <c r="N52" s="25"/>
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
       <c r="Q52" s="1"/>
@@ -3374,9 +3663,14 @@
       <c r="Z52" s="1"/>
       <c r="AA52" s="1"/>
       <c r="AB52" s="1"/>
-    </row>
-    <row r="53" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B53" s="11"/>
+      <c r="AC52" s="1"/>
+      <c r="AD52" s="1"/>
+    </row>
+    <row r="53" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B53" s="11">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
@@ -3388,7 +3682,7 @@
       <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="15"/>
-      <c r="N53" s="23"/>
+      <c r="N53" s="25"/>
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
@@ -3403,9 +3697,14 @@
       <c r="Z53" s="1"/>
       <c r="AA53" s="1"/>
       <c r="AB53" s="1"/>
-    </row>
-    <row r="54" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B54" s="11"/>
+      <c r="AC53" s="1"/>
+      <c r="AD53" s="1"/>
+    </row>
+    <row r="54" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B54" s="11">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
@@ -3417,7 +3716,7 @@
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="15"/>
-      <c r="N54" s="23"/>
+      <c r="N54" s="25"/>
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
@@ -3432,9 +3731,14 @@
       <c r="Z54" s="1"/>
       <c r="AA54" s="1"/>
       <c r="AB54" s="1"/>
-    </row>
-    <row r="55" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B55" s="11"/>
+      <c r="AC54" s="1"/>
+      <c r="AD54" s="1"/>
+    </row>
+    <row r="55" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B55" s="11">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
@@ -3446,7 +3750,7 @@
       <c r="K55" s="3"/>
       <c r="L55" s="3"/>
       <c r="M55" s="15"/>
-      <c r="N55" s="23"/>
+      <c r="N55" s="25"/>
       <c r="O55" s="1"/>
       <c r="P55" s="1"/>
       <c r="Q55" s="1"/>
@@ -3461,9 +3765,14 @@
       <c r="Z55" s="1"/>
       <c r="AA55" s="1"/>
       <c r="AB55" s="1"/>
-    </row>
-    <row r="56" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="B56" s="11"/>
+      <c r="AC55" s="1"/>
+      <c r="AD55" s="1"/>
+    </row>
+    <row r="56" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B56" s="11">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
@@ -3475,8 +3784,8 @@
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="15"/>
-      <c r="N56" s="23"/>
-      <c r="O56" s="1"/>
+      <c r="N56" s="25"/>
+      <c r="O56" s="20"/>
       <c r="P56" s="1"/>
       <c r="Q56" s="1"/>
       <c r="R56" s="1"/>
@@ -3490,8 +3799,10 @@
       <c r="Z56" s="1"/>
       <c r="AA56" s="1"/>
       <c r="AB56" s="1"/>
-    </row>
-    <row r="57" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="AC56" s="1"/>
+      <c r="AD56" s="1"/>
+    </row>
+    <row r="57" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B57" s="11"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
@@ -3520,9 +3831,11 @@
       <c r="AA57" s="1"/>
       <c r="AB57" s="1"/>
     </row>
-    <row r="58" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B58" s="11"/>
-      <c r="C58" s="3"/>
+      <c r="C58" s="21" t="s">
+        <v>43</v>
+      </c>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
@@ -3549,7 +3862,7 @@
       <c r="AA58" s="1"/>
       <c r="AB58" s="1"/>
     </row>
-    <row r="59" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B59" s="11"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
@@ -3578,7 +3891,7 @@
       <c r="AA59" s="1"/>
       <c r="AB59" s="1"/>
     </row>
-    <row r="60" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B60" s="11"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
@@ -3607,7 +3920,7 @@
       <c r="AA60" s="1"/>
       <c r="AB60" s="1"/>
     </row>
-    <row r="61" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B61" s="11"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
@@ -3636,7 +3949,7 @@
       <c r="AA61" s="1"/>
       <c r="AB61" s="1"/>
     </row>
-    <row r="62" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B62" s="11"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
@@ -3665,7 +3978,7 @@
       <c r="AA62" s="1"/>
       <c r="AB62" s="1"/>
     </row>
-    <row r="63" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B63" s="11"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
@@ -3694,7 +4007,7 @@
       <c r="AA63" s="1"/>
       <c r="AB63" s="1"/>
     </row>
-    <row r="64" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:30" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B64" s="11"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
@@ -31157,11 +31470,360 @@
       <c r="AA1010" s="1"/>
       <c r="AB1010" s="1"/>
     </row>
+    <row r="1011" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1011" s="11"/>
+      <c r="C1011" s="3"/>
+      <c r="D1011" s="3"/>
+      <c r="E1011" s="3"/>
+      <c r="F1011" s="3"/>
+      <c r="G1011" s="3"/>
+      <c r="H1011" s="3"/>
+      <c r="I1011" s="3"/>
+      <c r="J1011" s="3"/>
+      <c r="K1011" s="3"/>
+      <c r="L1011" s="3"/>
+      <c r="M1011" s="15"/>
+      <c r="N1011" s="23"/>
+      <c r="O1011" s="1"/>
+      <c r="P1011" s="1"/>
+      <c r="Q1011" s="1"/>
+      <c r="R1011" s="1"/>
+      <c r="S1011" s="1"/>
+      <c r="T1011" s="1"/>
+      <c r="U1011" s="1"/>
+      <c r="V1011" s="1"/>
+      <c r="W1011" s="1"/>
+      <c r="X1011" s="1"/>
+      <c r="Y1011" s="1"/>
+      <c r="Z1011" s="1"/>
+      <c r="AA1011" s="1"/>
+      <c r="AB1011" s="1"/>
+    </row>
+    <row r="1012" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1012" s="11"/>
+      <c r="C1012" s="3"/>
+      <c r="D1012" s="3"/>
+      <c r="E1012" s="3"/>
+      <c r="F1012" s="3"/>
+      <c r="G1012" s="3"/>
+      <c r="H1012" s="3"/>
+      <c r="I1012" s="3"/>
+      <c r="J1012" s="3"/>
+      <c r="K1012" s="3"/>
+      <c r="L1012" s="3"/>
+      <c r="M1012" s="15"/>
+      <c r="N1012" s="23"/>
+      <c r="O1012" s="1"/>
+      <c r="P1012" s="1"/>
+      <c r="Q1012" s="1"/>
+      <c r="R1012" s="1"/>
+      <c r="S1012" s="1"/>
+      <c r="T1012" s="1"/>
+      <c r="U1012" s="1"/>
+      <c r="V1012" s="1"/>
+      <c r="W1012" s="1"/>
+      <c r="X1012" s="1"/>
+      <c r="Y1012" s="1"/>
+      <c r="Z1012" s="1"/>
+      <c r="AA1012" s="1"/>
+      <c r="AB1012" s="1"/>
+    </row>
+    <row r="1013" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1013" s="11"/>
+      <c r="C1013" s="3"/>
+      <c r="D1013" s="3"/>
+      <c r="E1013" s="3"/>
+      <c r="F1013" s="3"/>
+      <c r="G1013" s="3"/>
+      <c r="H1013" s="3"/>
+      <c r="I1013" s="3"/>
+      <c r="J1013" s="3"/>
+      <c r="K1013" s="3"/>
+      <c r="L1013" s="3"/>
+      <c r="M1013" s="15"/>
+      <c r="N1013" s="23"/>
+      <c r="O1013" s="1"/>
+      <c r="P1013" s="1"/>
+      <c r="Q1013" s="1"/>
+      <c r="R1013" s="1"/>
+      <c r="S1013" s="1"/>
+      <c r="T1013" s="1"/>
+      <c r="U1013" s="1"/>
+      <c r="V1013" s="1"/>
+      <c r="W1013" s="1"/>
+      <c r="X1013" s="1"/>
+      <c r="Y1013" s="1"/>
+      <c r="Z1013" s="1"/>
+      <c r="AA1013" s="1"/>
+      <c r="AB1013" s="1"/>
+    </row>
+    <row r="1014" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1014" s="11"/>
+      <c r="C1014" s="3"/>
+      <c r="D1014" s="3"/>
+      <c r="E1014" s="3"/>
+      <c r="F1014" s="3"/>
+      <c r="G1014" s="3"/>
+      <c r="H1014" s="3"/>
+      <c r="I1014" s="3"/>
+      <c r="J1014" s="3"/>
+      <c r="K1014" s="3"/>
+      <c r="L1014" s="3"/>
+      <c r="M1014" s="15"/>
+      <c r="N1014" s="23"/>
+      <c r="O1014" s="1"/>
+      <c r="P1014" s="1"/>
+      <c r="Q1014" s="1"/>
+      <c r="R1014" s="1"/>
+      <c r="S1014" s="1"/>
+      <c r="T1014" s="1"/>
+      <c r="U1014" s="1"/>
+      <c r="V1014" s="1"/>
+      <c r="W1014" s="1"/>
+      <c r="X1014" s="1"/>
+      <c r="Y1014" s="1"/>
+      <c r="Z1014" s="1"/>
+      <c r="AA1014" s="1"/>
+      <c r="AB1014" s="1"/>
+    </row>
+    <row r="1015" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1015" s="11"/>
+      <c r="C1015" s="3"/>
+      <c r="D1015" s="3"/>
+      <c r="E1015" s="3"/>
+      <c r="F1015" s="3"/>
+      <c r="G1015" s="3"/>
+      <c r="H1015" s="3"/>
+      <c r="I1015" s="3"/>
+      <c r="J1015" s="3"/>
+      <c r="K1015" s="3"/>
+      <c r="L1015" s="3"/>
+      <c r="M1015" s="15"/>
+      <c r="N1015" s="23"/>
+      <c r="O1015" s="1"/>
+      <c r="P1015" s="1"/>
+      <c r="Q1015" s="1"/>
+      <c r="R1015" s="1"/>
+      <c r="S1015" s="1"/>
+      <c r="T1015" s="1"/>
+      <c r="U1015" s="1"/>
+      <c r="V1015" s="1"/>
+      <c r="W1015" s="1"/>
+      <c r="X1015" s="1"/>
+      <c r="Y1015" s="1"/>
+      <c r="Z1015" s="1"/>
+      <c r="AA1015" s="1"/>
+      <c r="AB1015" s="1"/>
+    </row>
+    <row r="1016" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1016" s="11"/>
+      <c r="C1016" s="3"/>
+      <c r="D1016" s="3"/>
+      <c r="E1016" s="3"/>
+      <c r="F1016" s="3"/>
+      <c r="G1016" s="3"/>
+      <c r="H1016" s="3"/>
+      <c r="I1016" s="3"/>
+      <c r="J1016" s="3"/>
+      <c r="K1016" s="3"/>
+      <c r="L1016" s="3"/>
+      <c r="M1016" s="15"/>
+      <c r="N1016" s="23"/>
+      <c r="O1016" s="1"/>
+      <c r="P1016" s="1"/>
+      <c r="Q1016" s="1"/>
+      <c r="R1016" s="1"/>
+      <c r="S1016" s="1"/>
+      <c r="T1016" s="1"/>
+      <c r="U1016" s="1"/>
+      <c r="V1016" s="1"/>
+      <c r="W1016" s="1"/>
+      <c r="X1016" s="1"/>
+      <c r="Y1016" s="1"/>
+      <c r="Z1016" s="1"/>
+      <c r="AA1016" s="1"/>
+      <c r="AB1016" s="1"/>
+    </row>
+    <row r="1017" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1017" s="11"/>
+      <c r="C1017" s="3"/>
+      <c r="D1017" s="3"/>
+      <c r="E1017" s="3"/>
+      <c r="F1017" s="3"/>
+      <c r="G1017" s="3"/>
+      <c r="H1017" s="3"/>
+      <c r="I1017" s="3"/>
+      <c r="J1017" s="3"/>
+      <c r="K1017" s="3"/>
+      <c r="L1017" s="3"/>
+      <c r="M1017" s="15"/>
+      <c r="N1017" s="23"/>
+      <c r="O1017" s="1"/>
+      <c r="P1017" s="1"/>
+      <c r="Q1017" s="1"/>
+      <c r="R1017" s="1"/>
+      <c r="S1017" s="1"/>
+      <c r="T1017" s="1"/>
+      <c r="U1017" s="1"/>
+      <c r="V1017" s="1"/>
+      <c r="W1017" s="1"/>
+      <c r="X1017" s="1"/>
+      <c r="Y1017" s="1"/>
+      <c r="Z1017" s="1"/>
+      <c r="AA1017" s="1"/>
+      <c r="AB1017" s="1"/>
+    </row>
+    <row r="1018" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1018" s="11"/>
+      <c r="C1018" s="3"/>
+      <c r="D1018" s="3"/>
+      <c r="E1018" s="3"/>
+      <c r="F1018" s="3"/>
+      <c r="G1018" s="3"/>
+      <c r="H1018" s="3"/>
+      <c r="I1018" s="3"/>
+      <c r="J1018" s="3"/>
+      <c r="K1018" s="3"/>
+      <c r="L1018" s="3"/>
+      <c r="M1018" s="15"/>
+      <c r="N1018" s="23"/>
+      <c r="O1018" s="1"/>
+      <c r="P1018" s="1"/>
+      <c r="Q1018" s="1"/>
+      <c r="R1018" s="1"/>
+      <c r="S1018" s="1"/>
+      <c r="T1018" s="1"/>
+      <c r="U1018" s="1"/>
+      <c r="V1018" s="1"/>
+      <c r="W1018" s="1"/>
+      <c r="X1018" s="1"/>
+      <c r="Y1018" s="1"/>
+      <c r="Z1018" s="1"/>
+      <c r="AA1018" s="1"/>
+      <c r="AB1018" s="1"/>
+    </row>
+    <row r="1019" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1019" s="11"/>
+      <c r="C1019" s="3"/>
+      <c r="D1019" s="3"/>
+      <c r="E1019" s="3"/>
+      <c r="F1019" s="3"/>
+      <c r="G1019" s="3"/>
+      <c r="H1019" s="3"/>
+      <c r="I1019" s="3"/>
+      <c r="J1019" s="3"/>
+      <c r="K1019" s="3"/>
+      <c r="L1019" s="3"/>
+      <c r="M1019" s="15"/>
+      <c r="N1019" s="23"/>
+      <c r="O1019" s="1"/>
+      <c r="P1019" s="1"/>
+      <c r="Q1019" s="1"/>
+      <c r="R1019" s="1"/>
+      <c r="S1019" s="1"/>
+      <c r="T1019" s="1"/>
+      <c r="U1019" s="1"/>
+      <c r="V1019" s="1"/>
+      <c r="W1019" s="1"/>
+      <c r="X1019" s="1"/>
+      <c r="Y1019" s="1"/>
+      <c r="Z1019" s="1"/>
+      <c r="AA1019" s="1"/>
+      <c r="AB1019" s="1"/>
+    </row>
+    <row r="1020" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1020" s="11"/>
+      <c r="C1020" s="3"/>
+      <c r="D1020" s="3"/>
+      <c r="E1020" s="3"/>
+      <c r="F1020" s="3"/>
+      <c r="G1020" s="3"/>
+      <c r="H1020" s="3"/>
+      <c r="I1020" s="3"/>
+      <c r="J1020" s="3"/>
+      <c r="K1020" s="3"/>
+      <c r="L1020" s="3"/>
+      <c r="M1020" s="15"/>
+      <c r="N1020" s="23"/>
+      <c r="O1020" s="1"/>
+      <c r="P1020" s="1"/>
+      <c r="Q1020" s="1"/>
+      <c r="R1020" s="1"/>
+      <c r="S1020" s="1"/>
+      <c r="T1020" s="1"/>
+      <c r="U1020" s="1"/>
+      <c r="V1020" s="1"/>
+      <c r="W1020" s="1"/>
+      <c r="X1020" s="1"/>
+      <c r="Y1020" s="1"/>
+      <c r="Z1020" s="1"/>
+      <c r="AA1020" s="1"/>
+      <c r="AB1020" s="1"/>
+    </row>
+    <row r="1021" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1021" s="11"/>
+      <c r="C1021" s="3"/>
+      <c r="D1021" s="3"/>
+      <c r="E1021" s="3"/>
+      <c r="F1021" s="3"/>
+      <c r="G1021" s="3"/>
+      <c r="H1021" s="3"/>
+      <c r="I1021" s="3"/>
+      <c r="J1021" s="3"/>
+      <c r="K1021" s="3"/>
+      <c r="L1021" s="3"/>
+      <c r="M1021" s="15"/>
+      <c r="N1021" s="23"/>
+      <c r="O1021" s="1"/>
+      <c r="P1021" s="1"/>
+      <c r="Q1021" s="1"/>
+      <c r="R1021" s="1"/>
+      <c r="S1021" s="1"/>
+      <c r="T1021" s="1"/>
+      <c r="U1021" s="1"/>
+      <c r="V1021" s="1"/>
+      <c r="W1021" s="1"/>
+      <c r="X1021" s="1"/>
+      <c r="Y1021" s="1"/>
+      <c r="Z1021" s="1"/>
+      <c r="AA1021" s="1"/>
+      <c r="AB1021" s="1"/>
+    </row>
+    <row r="1022" spans="2:28" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B1022" s="11"/>
+      <c r="C1022" s="3"/>
+      <c r="D1022" s="3"/>
+      <c r="E1022" s="3"/>
+      <c r="F1022" s="3"/>
+      <c r="G1022" s="3"/>
+      <c r="H1022" s="3"/>
+      <c r="I1022" s="3"/>
+      <c r="J1022" s="3"/>
+      <c r="K1022" s="3"/>
+      <c r="L1022" s="3"/>
+      <c r="M1022" s="15"/>
+      <c r="N1022" s="23"/>
+      <c r="O1022" s="1"/>
+      <c r="P1022" s="1"/>
+      <c r="Q1022" s="1"/>
+      <c r="R1022" s="1"/>
+      <c r="S1022" s="1"/>
+      <c r="T1022" s="1"/>
+      <c r="U1022" s="1"/>
+      <c r="V1022" s="1"/>
+      <c r="W1022" s="1"/>
+      <c r="X1022" s="1"/>
+      <c r="Y1022" s="1"/>
+      <c r="Z1022" s="1"/>
+      <c r="AA1022" s="1"/>
+      <c r="AB1022" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="H2:L2"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>